<commit_message>
ajout des compétences dans le tableau
</commit_message>
<xml_diff>
--- a/PDF/chetouani-competences.xlsx
+++ b/PDF/chetouani-competences.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chetouani\Documents\stage\Stage-main\Rapport de Stage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ayyoub\Documents\Portfolio\PDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA0236E8-163E-407E-96E9-F4A44EE64F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2B5049-7BA4-4343-8BAC-37140B109D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15216" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -498,7 +498,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -521,12 +521,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -563,15 +557,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -596,20 +605,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -920,81 +917,81 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ82"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.5546875" customWidth="1"/>
-    <col min="44" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.5703125" customWidth="1"/>
+    <col min="44" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:43" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="H1" s="22"/>
+    </row>
+    <row r="2" spans="1:43" ht="40.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="3" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+    </row>
+    <row r="3" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="33" t="s">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="34"/>
-      <c r="H3" s="35"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="25"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
+    <row r="4" spans="1:43" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="14" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+    <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="34" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="6" t="s">
@@ -1016,25 +1013,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:43" s="2" customFormat="1" ht="325.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="36" t="s">
+    <row r="6" spans="1:43" s="2" customFormat="1" ht="325.14999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="27"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="36" t="s">
         <v>14</v>
       </c>
       <c r="I6"/>
@@ -1073,17 +1070,17 @@
       <c r="AP6"/>
       <c r="AQ6"/>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A7" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="27"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="30"/>
       <c r="I7"/>
       <c r="J7"/>
       <c r="K7"/>
@@ -1120,19 +1117,23 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="21">
         <v>45778</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="19"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16">
+        <v>3</v>
+      </c>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16">
+        <v>2</v>
+      </c>
+      <c r="H8" s="17"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1169,19 +1170,21 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="21">
         <v>45931</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="19"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16">
+        <v>2</v>
+      </c>
+      <c r="H9" s="17"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1218,19 +1221,21 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="19"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16">
+        <v>2</v>
+      </c>
+      <c r="H10" s="17"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1267,19 +1272,19 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="19"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="17"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1316,19 +1321,21 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="19"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16">
+        <v>2</v>
+      </c>
+      <c r="H12" s="17"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1365,15 +1372,15 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1410,15 +1417,15 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="19"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="17"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1455,15 +1462,15 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="19"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="17"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1500,15 +1507,15 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="19"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="17"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1545,15 +1552,15 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="19"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1590,17 +1597,17 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A18" s="28" t="s">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A18" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="30"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="33"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1637,18 +1644,18 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="19"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="17"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1685,15 +1692,15 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1730,15 +1737,15 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="19"/>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="9"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="17"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1775,15 +1782,15 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="19"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="9"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1820,15 +1827,15 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="19"/>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="9"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1865,15 +1872,15 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="19"/>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="9"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="17"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -1910,15 +1917,15 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="19"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="17"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -1955,15 +1962,15 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="19"/>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="9"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2000,17 +2007,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A27" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="30"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="33"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2047,17 +2054,19 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="19"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16">
+        <v>2</v>
+      </c>
+      <c r="H28" s="17"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2094,15 +2103,15 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="19"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="9"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2139,15 +2148,15 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="19"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="9"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2184,15 +2193,15 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="11"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="19"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="9"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="17"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2229,15 +2238,15 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="11"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="19"/>
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="9"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="17"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2274,15 +2283,15 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="19"/>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="9"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="17"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2319,15 +2328,15 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="19"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="9"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="17"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2364,15 +2373,15 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="12"/>
-      <c r="B35" s="13"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="21"/>
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="10"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="19"/>
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
@@ -2409,7 +2418,7 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="5"/>
       <c r="B36" s="3"/>
       <c r="C36" s="4"/>
@@ -2454,65 +2463,65 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="82" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B5:B6"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
tableau de compétence modifié
</commit_message>
<xml_diff>
--- a/PDF/chetouani-competences.xlsx
+++ b/PDF/chetouani-competences.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ayyoub\Documents\Portfolio\PDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2B5049-7BA4-4343-8BAC-37140B109D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC57150E-2536-4DB5-AAA7-66E5A427B4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -557,9 +557,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -605,8 +602,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -927,56 +927,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="21"/>
     </row>
     <row r="2" spans="1:43" ht="40.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="23" t="s">
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="25"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="24"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="25"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
       <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
@@ -988,10 +988,10 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="33" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="6" t="s">
@@ -1014,21 +1014,21 @@
       </c>
     </row>
     <row r="6" spans="1:43" s="2" customFormat="1" ht="325.14999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27"/>
-      <c r="B6" s="35"/>
-      <c r="C6" s="20" t="s">
+      <c r="A6" s="26"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="35" t="s">
         <v>13</v>
       </c>
       <c r="H6" s="36" t="s">
@@ -1071,16 +1071,16 @@
       <c r="AQ6"/>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="29"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="30"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="29"/>
       <c r="I7"/>
       <c r="J7"/>
       <c r="K7"/>
@@ -1121,7 +1121,7 @@
       <c r="A8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="20">
         <v>45778</v>
       </c>
       <c r="C8" s="15"/>
@@ -1174,7 +1174,7 @@
       <c r="A9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="20">
         <v>45931</v>
       </c>
       <c r="C9" s="16"/>
@@ -1598,16 +1598,16 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="33"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="32"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -2008,16 +2008,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="33"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="32"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>

</xml_diff>

<commit_message>
tableau de compétence complété
</commit_message>
<xml_diff>
--- a/PDF/chetouani-competences.xlsx
+++ b/PDF/chetouani-competences.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ayyoub\Documents\Portfolio\PDF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chetouani\Documents\Portfolio\PDF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC57150E-2536-4DB5-AAA7-66E5A427B4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{155EA6CE-9E80-4FA5-A44C-8EA52BC52FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>mars-avril 2026</t>
+  </si>
+  <si>
+    <t>2, 3</t>
   </si>
 </sst>
 </file>
@@ -560,9 +563,45 @@
     <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -571,42 +610,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -917,66 +920,66 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ82"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.5703125" customWidth="1"/>
-    <col min="44" max="16384" width="10.7109375" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.5546875" customWidth="1"/>
+    <col min="44" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="21"/>
-    </row>
-    <row r="2" spans="1:43" ht="40.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:43" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-    </row>
-    <row r="3" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="3" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="22" t="s">
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="24"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="36"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+    <row r="4" spans="1:43" ht="40.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="24"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
       <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
@@ -987,11 +990,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="25" t="s">
+    <row r="5" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="32" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="6" t="s">
@@ -1013,25 +1016,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:43" s="2" customFormat="1" ht="325.14999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="26"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="35" t="s">
+    <row r="6" spans="1:43" s="2" customFormat="1" ht="325.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="24"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="35" t="s">
+      <c r="F6" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="35" t="s">
+      <c r="G6" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="22" t="s">
         <v>14</v>
       </c>
       <c r="I6"/>
@@ -1070,17 +1073,17 @@
       <c r="AP6"/>
       <c r="AQ6"/>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A7" s="27" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="29"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="28"/>
       <c r="I7"/>
       <c r="J7"/>
       <c r="K7"/>
@@ -1117,7 +1120,7 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>26</v>
       </c>
@@ -1129,7 +1132,9 @@
       <c r="E8" s="16">
         <v>3</v>
       </c>
-      <c r="F8" s="16"/>
+      <c r="F8" s="16">
+        <v>3</v>
+      </c>
       <c r="G8" s="16">
         <v>2</v>
       </c>
@@ -1170,7 +1175,7 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>29</v>
       </c>
@@ -1179,7 +1184,9 @@
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
+      <c r="E9" s="16">
+        <v>3</v>
+      </c>
       <c r="F9" s="16"/>
       <c r="G9" s="16">
         <v>2</v>
@@ -1221,17 +1228,21 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="16"/>
+      <c r="C10" s="16">
+        <v>3</v>
+      </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
+      <c r="F10" s="16" t="s">
+        <v>37</v>
+      </c>
       <c r="G10" s="16">
         <v>2</v>
       </c>
@@ -1272,7 +1283,7 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>31</v>
       </c>
@@ -1280,9 +1291,13 @@
         <v>35</v>
       </c>
       <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
+      <c r="D11" s="16">
+        <v>3</v>
+      </c>
       <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
+      <c r="F11" s="16" t="s">
+        <v>37</v>
+      </c>
       <c r="G11" s="16"/>
       <c r="H11" s="17"/>
       <c r="I11"/>
@@ -1321,7 +1336,7 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>33</v>
       </c>
@@ -1335,7 +1350,9 @@
       <c r="G12" s="16">
         <v>2</v>
       </c>
-      <c r="H12" s="17"/>
+      <c r="H12" s="17">
+        <v>1</v>
+      </c>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1372,7 +1389,7 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="8"/>
       <c r="C13" s="16"/>
@@ -1417,7 +1434,7 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
       <c r="B14" s="8"/>
       <c r="C14" s="16"/>
@@ -1462,7 +1479,7 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9"/>
       <c r="B15" s="8"/>
       <c r="C15" s="16"/>
@@ -1507,7 +1524,7 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
       <c r="B16" s="8"/>
       <c r="C16" s="16"/>
@@ -1552,7 +1569,7 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="B17" s="8"/>
       <c r="C17" s="16"/>
@@ -1597,17 +1614,17 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A18" s="30" t="s">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A18" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="32"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="31"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1644,7 +1661,7 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>27</v>
       </c>
@@ -1654,7 +1671,9 @@
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
+      <c r="G19" s="16">
+        <v>2</v>
+      </c>
       <c r="H19" s="17"/>
       <c r="I19"/>
       <c r="J19"/>
@@ -1692,7 +1711,7 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="B20" s="8"/>
       <c r="C20" s="16"/>
@@ -1737,7 +1756,7 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="8"/>
       <c r="C21" s="16"/>
@@ -1782,7 +1801,7 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="8"/>
       <c r="C22" s="16"/>
@@ -1827,7 +1846,7 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="8"/>
       <c r="C23" s="16"/>
@@ -1872,7 +1891,7 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="8"/>
       <c r="C24" s="16"/>
@@ -1917,7 +1936,7 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="8"/>
       <c r="C25" s="16"/>
@@ -1962,7 +1981,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="B26" s="8"/>
       <c r="C26" s="16"/>
@@ -2007,17 +2026,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="30" t="s">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A27" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="32"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="31"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2054,13 +2073,17 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="8"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
+      <c r="C28" s="16">
+        <v>2</v>
+      </c>
+      <c r="D28" s="16">
+        <v>2</v>
+      </c>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
       <c r="G28" s="16">
@@ -2103,7 +2126,7 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="B29" s="8"/>
       <c r="C29" s="16"/>
@@ -2148,7 +2171,7 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="B30" s="8"/>
       <c r="C30" s="16"/>
@@ -2193,7 +2216,7 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
       <c r="B31" s="8"/>
       <c r="C31" s="16"/>
@@ -2238,7 +2261,7 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="8"/>
       <c r="C32" s="16"/>
@@ -2283,7 +2306,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="8"/>
       <c r="C33" s="16"/>
@@ -2328,7 +2351,7 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
       <c r="B34" s="8"/>
       <c r="C34" s="16"/>
@@ -2373,7 +2396,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10"/>
       <c r="B35" s="11"/>
       <c r="C35" s="18"/>
@@ -2418,7 +2441,7 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
       <c r="B36" s="3"/>
       <c r="C36" s="4"/>
@@ -2463,65 +2486,65 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="82" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>